<commit_message>
fix: aggiunta in output riserva d'ufficio
</commit_message>
<xml_diff>
--- a/src/output-files-generator/Template output _Giornata N - Girone X.xlsx
+++ b/src/output-files-generator/Template output _Giornata N - Girone X.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Shared/progetti/personal/fife-cup-matches-calculator/src/output-files-generator/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liusdellapietal/progetti personal/fife-cup-matches-calculator/src/output-files-generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D801EC-69CB-AA42-82AE-DD86F7B78906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7224A709-D9FB-484F-9F97-333F8841AB95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="25720" windowHeight="15940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="25720" windowHeight="15940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Formazioni giornata" sheetId="2" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="19">
   <si>
     <t>Panchina</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t>diff &gt;= 8</t>
+  </si>
+  <si>
+    <t>Riserva d'ufficio</t>
   </si>
 </sst>
 </file>
@@ -343,7 +346,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -382,16 +385,7 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -404,12 +398,16 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -418,11 +416,17 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1565,71 +1569,71 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AD3DEF5-60E5-BD4E-ACCC-BBFBF84A9848}">
-  <dimension ref="A1:U56"/>
+  <dimension ref="A1:U58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="47"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="34"/>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="40"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="37"/>
       <c r="F3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="36" t="s">
+      <c r="G3" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="37"/>
-      <c r="I3" s="38"/>
-      <c r="J3" s="39"/>
-      <c r="K3" s="40"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="37"/>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="44"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="3"/>
-      <c r="G4" s="45" t="s">
+      <c r="G4" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="35"/>
-      <c r="I4" s="42"/>
-      <c r="J4" s="43"/>
-      <c r="K4" s="43"/>
-      <c r="N4" s="48" t="s">
+      <c r="H4" s="30"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="40"/>
+      <c r="K4" s="40"/>
+      <c r="N4" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="O4" s="48"/>
-      <c r="P4" s="48"/>
-      <c r="Q4" s="48" t="s">
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="R4" s="48"/>
-      <c r="S4" s="48"/>
-      <c r="T4" s="48"/>
-      <c r="U4" s="48"/>
+      <c r="R4" s="24"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="24"/>
+      <c r="U4" s="24"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" s="4"/>
@@ -1643,20 +1647,20 @@
       <c r="I5" s="4"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
-      <c r="N5" s="48">
+      <c r="N5" s="24">
         <f>SUM(D9:D12)</f>
         <v>0</v>
       </c>
-      <c r="O5" s="48"/>
-      <c r="P5" s="48"/>
-      <c r="Q5" s="48">
+      <c r="O5" s="24"/>
+      <c r="P5" s="24"/>
+      <c r="Q5" s="24">
         <f>SUM(J9:J12)</f>
         <v>0</v>
       </c>
-      <c r="R5" s="48"/>
-      <c r="S5" s="48"/>
-      <c r="T5" s="48"/>
-      <c r="U5" s="48"/>
+      <c r="R5" s="24"/>
+      <c r="S5" s="24"/>
+      <c r="T5" s="24"/>
+      <c r="U5" s="24"/>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" s="6"/>
@@ -1670,14 +1674,14 @@
       <c r="I6" s="6"/>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>
-      <c r="N6" s="48"/>
-      <c r="O6" s="48"/>
-      <c r="P6" s="48"/>
-      <c r="Q6" s="48"/>
-      <c r="R6" s="48"/>
-      <c r="S6" s="48"/>
-      <c r="T6" s="48"/>
-      <c r="U6" s="48"/>
+      <c r="N6" s="24"/>
+      <c r="O6" s="24"/>
+      <c r="P6" s="24"/>
+      <c r="Q6" s="24"/>
+      <c r="R6" s="24"/>
+      <c r="S6" s="24"/>
+      <c r="T6" s="24"/>
+      <c r="U6" s="24"/>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" s="6"/>
@@ -1691,14 +1695,14 @@
       <c r="I7" s="6"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="N7" s="48"/>
-      <c r="O7" s="48"/>
-      <c r="P7" s="48"/>
-      <c r="Q7" s="48"/>
-      <c r="R7" s="48"/>
-      <c r="S7" s="48"/>
-      <c r="T7" s="48"/>
-      <c r="U7" s="48"/>
+      <c r="N7" s="24"/>
+      <c r="O7" s="24"/>
+      <c r="P7" s="24"/>
+      <c r="Q7" s="24"/>
+      <c r="R7" s="24"/>
+      <c r="S7" s="24"/>
+      <c r="T7" s="24"/>
+      <c r="U7" s="24"/>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" s="6"/>
@@ -1712,18 +1716,18 @@
       <c r="I8" s="6"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
-      <c r="N8" s="48" t="s">
+      <c r="N8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="O8" s="48"/>
-      <c r="P8" s="48"/>
-      <c r="Q8" s="48" t="s">
+      <c r="O8" s="24"/>
+      <c r="P8" s="24"/>
+      <c r="Q8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="R8" s="48"/>
-      <c r="S8" s="48"/>
-      <c r="T8" s="48"/>
-      <c r="U8" s="48"/>
+      <c r="R8" s="24"/>
+      <c r="S8" s="24"/>
+      <c r="T8" s="24"/>
+      <c r="U8" s="24"/>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" s="6"/>
@@ -1737,22 +1741,22 @@
       <c r="I9" s="6"/>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
-      <c r="N9" s="48">
+      <c r="N9" s="24">
         <f>N5-Q5</f>
         <v>0</v>
       </c>
-      <c r="O9" s="48"/>
-      <c r="P9" s="48"/>
-      <c r="Q9" s="48">
+      <c r="O9" s="24"/>
+      <c r="P9" s="24"/>
+      <c r="Q9" s="24">
         <f>Q5-N5</f>
         <v>0</v>
       </c>
-      <c r="R9" s="48"/>
-      <c r="S9" s="48" t="s">
+      <c r="R9" s="24"/>
+      <c r="S9" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="T9" s="48"/>
-      <c r="U9" s="48">
+      <c r="T9" s="24"/>
+      <c r="U9" s="24">
         <v>2</v>
       </c>
     </row>
@@ -1768,16 +1772,16 @@
       <c r="I10" s="6"/>
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
-      <c r="N10" s="48"/>
-      <c r="O10" s="48"/>
-      <c r="P10" s="48"/>
-      <c r="Q10" s="48"/>
-      <c r="R10" s="48"/>
-      <c r="S10" s="48" t="s">
+      <c r="N10" s="24"/>
+      <c r="O10" s="24"/>
+      <c r="P10" s="24"/>
+      <c r="Q10" s="24"/>
+      <c r="R10" s="24"/>
+      <c r="S10" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="T10" s="48"/>
-      <c r="U10" s="48">
+      <c r="T10" s="24"/>
+      <c r="U10" s="24">
         <v>3</v>
       </c>
     </row>
@@ -1793,16 +1797,16 @@
       <c r="I11" s="6"/>
       <c r="J11" s="7"/>
       <c r="K11" s="7"/>
-      <c r="N11" s="48"/>
-      <c r="O11" s="48"/>
-      <c r="P11" s="48"/>
-      <c r="Q11" s="48"/>
-      <c r="R11" s="48"/>
-      <c r="S11" s="48" t="s">
+      <c r="N11" s="24"/>
+      <c r="O11" s="24"/>
+      <c r="P11" s="24"/>
+      <c r="Q11" s="24"/>
+      <c r="R11" s="24"/>
+      <c r="S11" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="T11" s="48"/>
-      <c r="U11" s="48">
+      <c r="T11" s="24"/>
+      <c r="U11" s="24">
         <v>4</v>
       </c>
     </row>
@@ -1859,23 +1863,23 @@
       <c r="K15" s="10"/>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="31"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="33"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="28"/>
       <c r="F16" s="11"/>
-      <c r="G16" s="34" t="s">
+      <c r="G16" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="H16" s="31"/>
-      <c r="I16" s="31"/>
-      <c r="J16" s="32"/>
-      <c r="K16" s="35"/>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="H16" s="26"/>
+      <c r="I16" s="26"/>
+      <c r="J16" s="27"/>
+      <c r="K16" s="30"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="12"/>
       <c r="B17" s="12"/>
       <c r="C17" s="4"/>
@@ -1888,7 +1892,7 @@
       <c r="J17" s="14"/>
       <c r="K17" s="14"/>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="15"/>
       <c r="B18" s="15"/>
       <c r="C18" s="6"/>
@@ -1901,7 +1905,7 @@
       <c r="J18" s="17"/>
       <c r="K18" s="17"/>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="15"/>
       <c r="B19" s="15"/>
       <c r="C19" s="6"/>
@@ -1914,7 +1918,7 @@
       <c r="J19" s="17"/>
       <c r="K19" s="17"/>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="15"/>
       <c r="B20" s="15"/>
       <c r="C20" s="6"/>
@@ -1927,7 +1931,7 @@
       <c r="J20" s="17"/>
       <c r="K20" s="17"/>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="15"/>
       <c r="B21" s="15"/>
       <c r="C21" s="6"/>
@@ -1940,7 +1944,7 @@
       <c r="J21" s="17"/>
       <c r="K21" s="17"/>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="15"/>
       <c r="B22" s="15"/>
       <c r="C22" s="6"/>
@@ -1953,7 +1957,7 @@
       <c r="J22" s="16"/>
       <c r="K22" s="16"/>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="15"/>
       <c r="B23" s="15"/>
       <c r="C23" s="6"/>
@@ -1966,7 +1970,7 @@
       <c r="J23" s="16"/>
       <c r="K23" s="16"/>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="18"/>
       <c r="B24" s="18"/>
       <c r="C24" s="9"/>
@@ -1979,163 +1983,161 @@
       <c r="J24" s="19"/>
       <c r="K24" s="19"/>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A25" s="27" t="s">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A25" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B25" s="28"/>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
+      <c r="B25" s="44"/>
+      <c r="C25" s="44"/>
+      <c r="D25" s="44"/>
       <c r="E25" s="20"/>
       <c r="F25" s="11"/>
-      <c r="G25" s="27" t="s">
+      <c r="G25" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="H25" s="28"/>
-      <c r="I25" s="28"/>
-      <c r="J25" s="28"/>
+      <c r="H25" s="44"/>
+      <c r="I25" s="44"/>
+      <c r="J25" s="44"/>
       <c r="K25" s="20"/>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A26" s="29" t="s">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="B26" s="28"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
+      <c r="B26" s="44"/>
+      <c r="C26" s="44"/>
+      <c r="D26" s="44"/>
       <c r="E26" s="21"/>
       <c r="F26" s="11"/>
-      <c r="G26" s="29" t="s">
+      <c r="G26" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="H26" s="28"/>
-      <c r="I26" s="28"/>
-      <c r="J26" s="28"/>
+      <c r="H26" s="44"/>
+      <c r="I26" s="44"/>
+      <c r="J26" s="44"/>
       <c r="K26" s="21"/>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A27" s="27" t="s">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A27" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="B27" s="28"/>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
+      <c r="B27" s="44"/>
+      <c r="C27" s="44"/>
+      <c r="D27" s="44"/>
       <c r="E27" s="20"/>
       <c r="F27" s="11"/>
-      <c r="G27" s="27" t="s">
+      <c r="G27" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="H27" s="28"/>
-      <c r="I27" s="28"/>
-      <c r="J27" s="28"/>
+      <c r="H27" s="44"/>
+      <c r="I27" s="44"/>
+      <c r="J27" s="44"/>
       <c r="K27" s="20"/>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A28" s="24" t="s">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A28" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="B28" s="44"/>
+      <c r="C28" s="44"/>
+      <c r="D28" s="44"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="H28" s="44"/>
+      <c r="I28" s="44"/>
+      <c r="J28" s="44"/>
+      <c r="K28" s="20"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A29" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="22"/>
-      <c r="G28" s="24" t="s">
+      <c r="B29" s="46"/>
+      <c r="C29" s="46"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="47"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="H28" s="25"/>
-      <c r="I28" s="25"/>
-      <c r="J28" s="25"/>
-      <c r="K28" s="26"/>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A31" s="36" t="s">
+      <c r="H29" s="46"/>
+      <c r="I29" s="46"/>
+      <c r="J29" s="46"/>
+      <c r="K29" s="47"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A32" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="B31" s="37"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="39"/>
-      <c r="E31" s="40"/>
-      <c r="F31" s="2" t="s">
+      <c r="B32" s="36"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="37"/>
+      <c r="F32" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G31" s="36" t="s">
+      <c r="G32" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="H31" s="37"/>
-      <c r="I31" s="38"/>
-      <c r="J31" s="39"/>
-      <c r="K31" s="40"/>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A32" s="41" t="s">
+      <c r="H32" s="36"/>
+      <c r="I32" s="32"/>
+      <c r="J32" s="33"/>
+      <c r="K32" s="37"/>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A33" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="B32" s="35"/>
-      <c r="C32" s="42"/>
-      <c r="D32" s="43"/>
-      <c r="E32" s="44"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="45" t="s">
+      <c r="B33" s="30"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="40"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="H32" s="35"/>
-      <c r="I32" s="42"/>
-      <c r="J32" s="43"/>
-      <c r="K32" s="43"/>
-      <c r="N32" s="48" t="s">
+      <c r="H33" s="30"/>
+      <c r="I33" s="39"/>
+      <c r="J33" s="40"/>
+      <c r="K33" s="40"/>
+      <c r="N33" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="O32" s="48"/>
-      <c r="P32" s="48"/>
-      <c r="Q32" s="48" t="s">
+      <c r="O33" s="24"/>
+      <c r="P33" s="24"/>
+      <c r="Q33" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="R32" s="48"/>
-      <c r="S32" s="48"/>
-    </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A33" s="4"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="1"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="5"/>
-      <c r="K33" s="5"/>
-      <c r="N33" s="48">
-        <f>SUM(D37:D40)</f>
+      <c r="R33" s="24"/>
+      <c r="S33" s="24"/>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="5"/>
+      <c r="N34" s="24">
+        <f>SUM(D38:D41)</f>
         <v>0</v>
       </c>
-      <c r="O33" s="48"/>
-      <c r="P33" s="48"/>
-      <c r="Q33" s="48">
-        <f>SUM(J37:J40)</f>
+      <c r="O34" s="24"/>
+      <c r="P34" s="24"/>
+      <c r="Q34" s="24">
+        <f>SUM(J38:J41)</f>
         <v>0</v>
       </c>
-      <c r="R33" s="48"/>
-      <c r="S33" s="48"/>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A34" s="6"/>
-      <c r="B34" s="6"/>
-      <c r="C34" s="6"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="6"/>
-      <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="7"/>
-      <c r="K34" s="7"/>
-      <c r="N34" s="48"/>
-      <c r="O34" s="48"/>
-      <c r="P34" s="48"/>
-      <c r="Q34" s="48"/>
-      <c r="R34" s="48"/>
-      <c r="S34" s="48"/>
+      <c r="R34" s="24"/>
+      <c r="S34" s="24"/>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A35" s="6"/>
@@ -2144,17 +2146,17 @@
       <c r="D35" s="7"/>
       <c r="E35" s="7"/>
       <c r="F35" s="8"/>
-      <c r="G35" s="15"/>
-      <c r="H35" s="15"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
       <c r="I35" s="6"/>
-      <c r="J35" s="16"/>
-      <c r="K35" s="16"/>
-      <c r="N35" s="48"/>
-      <c r="O35" s="48"/>
-      <c r="P35" s="48"/>
-      <c r="Q35" s="48"/>
-      <c r="R35" s="48"/>
-      <c r="S35" s="48"/>
+      <c r="J35" s="7"/>
+      <c r="K35" s="7"/>
+      <c r="N35" s="24"/>
+      <c r="O35" s="24"/>
+      <c r="P35" s="24"/>
+      <c r="Q35" s="24"/>
+      <c r="R35" s="24"/>
+      <c r="S35" s="24"/>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A36" s="6"/>
@@ -2163,21 +2165,17 @@
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
       <c r="F36" s="8"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
       <c r="I36" s="6"/>
-      <c r="J36" s="7"/>
-      <c r="K36" s="7"/>
-      <c r="N36" s="48" t="s">
-        <v>14</v>
-      </c>
-      <c r="O36" s="48"/>
-      <c r="P36" s="48"/>
-      <c r="Q36" s="48" t="s">
-        <v>14</v>
-      </c>
-      <c r="R36" s="48"/>
-      <c r="S36" s="48"/>
+      <c r="J36" s="16"/>
+      <c r="K36" s="16"/>
+      <c r="N36" s="24"/>
+      <c r="O36" s="24"/>
+      <c r="P36" s="24"/>
+      <c r="Q36" s="24"/>
+      <c r="R36" s="24"/>
+      <c r="S36" s="24"/>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A37" s="6"/>
@@ -2191,20 +2189,16 @@
       <c r="I37" s="6"/>
       <c r="J37" s="7"/>
       <c r="K37" s="7"/>
-      <c r="N37" s="48">
-        <f>N33-Q33</f>
-        <v>0</v>
-      </c>
-      <c r="O37" s="48"/>
-      <c r="P37" s="48"/>
-      <c r="Q37" s="48">
-        <f>Q33-N33</f>
-        <v>0</v>
-      </c>
-      <c r="R37" s="48"/>
-      <c r="S37" s="48" t="s">
-        <v>15</v>
-      </c>
+      <c r="N37" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="O37" s="24"/>
+      <c r="P37" s="24"/>
+      <c r="Q37" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="R37" s="24"/>
+      <c r="S37" s="24"/>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A38" s="6"/>
@@ -2218,13 +2212,19 @@
       <c r="I38" s="6"/>
       <c r="J38" s="7"/>
       <c r="K38" s="7"/>
-      <c r="N38" s="48"/>
-      <c r="O38" s="48"/>
-      <c r="P38" s="48"/>
-      <c r="Q38" s="48"/>
-      <c r="R38" s="48"/>
-      <c r="S38" s="48" t="s">
-        <v>16</v>
+      <c r="N38" s="24">
+        <f>N34-Q34</f>
+        <v>0</v>
+      </c>
+      <c r="O38" s="24"/>
+      <c r="P38" s="24"/>
+      <c r="Q38" s="24">
+        <f>Q34-N34</f>
+        <v>0</v>
+      </c>
+      <c r="R38" s="24"/>
+      <c r="S38" s="24" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.2">
@@ -2239,13 +2239,13 @@
       <c r="I39" s="6"/>
       <c r="J39" s="7"/>
       <c r="K39" s="7"/>
-      <c r="N39" s="48"/>
-      <c r="O39" s="48"/>
-      <c r="P39" s="48"/>
-      <c r="Q39" s="48"/>
-      <c r="R39" s="48"/>
-      <c r="S39" s="48" t="s">
-        <v>17</v>
+      <c r="N39" s="24"/>
+      <c r="O39" s="24"/>
+      <c r="P39" s="24"/>
+      <c r="Q39" s="24"/>
+      <c r="R39" s="24"/>
+      <c r="S39" s="24" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.2">
@@ -2260,6 +2260,14 @@
       <c r="I40" s="6"/>
       <c r="J40" s="7"/>
       <c r="K40" s="7"/>
+      <c r="N40" s="24"/>
+      <c r="O40" s="24"/>
+      <c r="P40" s="24"/>
+      <c r="Q40" s="24"/>
+      <c r="R40" s="24"/>
+      <c r="S40" s="24" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A41" s="6"/>
@@ -2281,93 +2289,93 @@
       <c r="D42" s="7"/>
       <c r="E42" s="7"/>
       <c r="F42" s="8"/>
-      <c r="G42" s="15"/>
-      <c r="H42" s="15"/>
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
       <c r="I42" s="6"/>
-      <c r="J42" s="16"/>
-      <c r="K42" s="16"/>
+      <c r="J42" s="7"/>
+      <c r="K42" s="7"/>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A43" s="9"/>
-      <c r="B43" s="9"/>
-      <c r="C43" s="9"/>
-      <c r="D43" s="10"/>
-      <c r="E43" s="10"/>
+      <c r="A43" s="6"/>
+      <c r="B43" s="6"/>
+      <c r="C43" s="6"/>
+      <c r="D43" s="7"/>
+      <c r="E43" s="7"/>
       <c r="F43" s="8"/>
-      <c r="G43" s="9"/>
-      <c r="H43" s="9"/>
-      <c r="I43" s="9"/>
-      <c r="J43" s="10"/>
-      <c r="K43" s="10"/>
+      <c r="G43" s="15"/>
+      <c r="H43" s="15"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="16"/>
+      <c r="K43" s="16"/>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A44" s="30" t="s">
+      <c r="A44" s="9"/>
+      <c r="B44" s="9"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="8"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
+      <c r="I44" s="9"/>
+      <c r="J44" s="10"/>
+      <c r="K44" s="10"/>
+    </row>
+    <row r="45" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A45" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B44" s="31"/>
-      <c r="C44" s="31"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="33"/>
-      <c r="F44" s="11"/>
-      <c r="G44" s="34" t="s">
+      <c r="B45" s="26"/>
+      <c r="C45" s="26"/>
+      <c r="D45" s="27"/>
+      <c r="E45" s="28"/>
+      <c r="F45" s="11"/>
+      <c r="G45" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="H44" s="31"/>
-      <c r="I44" s="31"/>
-      <c r="J44" s="32"/>
-      <c r="K44" s="35"/>
-    </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A45" s="12"/>
-      <c r="B45" s="12"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="13"/>
-      <c r="F45" s="8"/>
-      <c r="G45" s="12"/>
-      <c r="H45" s="12"/>
-      <c r="I45" s="4"/>
-      <c r="J45" s="14"/>
-      <c r="K45" s="14"/>
+      <c r="H45" s="26"/>
+      <c r="I45" s="26"/>
+      <c r="J45" s="27"/>
+      <c r="K45" s="30"/>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A46" s="15"/>
-      <c r="B46" s="15"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="17"/>
-      <c r="E46" s="17"/>
+      <c r="A46" s="12"/>
+      <c r="B46" s="12"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="13"/>
       <c r="F46" s="8"/>
-      <c r="G46" s="6"/>
-      <c r="H46" s="6"/>
-      <c r="I46" s="6"/>
-      <c r="J46" s="7"/>
-      <c r="K46" s="7"/>
+      <c r="G46" s="12"/>
+      <c r="H46" s="12"/>
+      <c r="I46" s="4"/>
+      <c r="J46" s="14"/>
+      <c r="K46" s="14"/>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A47" s="15"/>
       <c r="B47" s="15"/>
       <c r="C47" s="6"/>
-      <c r="D47" s="16"/>
-      <c r="E47" s="16"/>
+      <c r="D47" s="17"/>
+      <c r="E47" s="17"/>
       <c r="F47" s="8"/>
-      <c r="G47" s="15"/>
-      <c r="H47" s="15"/>
+      <c r="G47" s="6"/>
+      <c r="H47" s="6"/>
       <c r="I47" s="6"/>
-      <c r="J47" s="17"/>
-      <c r="K47" s="17"/>
+      <c r="J47" s="7"/>
+      <c r="K47" s="7"/>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A48" s="15"/>
       <c r="B48" s="15"/>
       <c r="C48" s="6"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="17"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="16"/>
       <c r="F48" s="8"/>
       <c r="G48" s="15"/>
       <c r="H48" s="15"/>
       <c r="I48" s="6"/>
-      <c r="J48" s="16"/>
-      <c r="K48" s="16"/>
+      <c r="J48" s="17"/>
+      <c r="K48" s="17"/>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" s="15"/>
@@ -2379,21 +2387,21 @@
       <c r="G49" s="15"/>
       <c r="H49" s="15"/>
       <c r="I49" s="6"/>
-      <c r="J49" s="17"/>
-      <c r="K49" s="17"/>
+      <c r="J49" s="16"/>
+      <c r="K49" s="16"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" s="15"/>
       <c r="B50" s="15"/>
       <c r="C50" s="6"/>
-      <c r="D50" s="16"/>
-      <c r="E50" s="16"/>
+      <c r="D50" s="17"/>
+      <c r="E50" s="17"/>
       <c r="F50" s="8"/>
       <c r="G50" s="15"/>
       <c r="H50" s="15"/>
       <c r="I50" s="6"/>
-      <c r="J50" s="16"/>
-      <c r="K50" s="16"/>
+      <c r="J50" s="17"/>
+      <c r="K50" s="17"/>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" s="15"/>
@@ -2409,88 +2417,144 @@
       <c r="K51" s="16"/>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A52" s="18"/>
-      <c r="B52" s="18"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="23"/>
-      <c r="E52" s="23"/>
+      <c r="A52" s="15"/>
+      <c r="B52" s="15"/>
+      <c r="C52" s="6"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="16"/>
       <c r="F52" s="8"/>
-      <c r="G52" s="9"/>
-      <c r="H52" s="9"/>
-      <c r="I52" s="9"/>
-      <c r="J52" s="10"/>
-      <c r="K52" s="10"/>
+      <c r="G52" s="15"/>
+      <c r="H52" s="15"/>
+      <c r="I52" s="6"/>
+      <c r="J52" s="16"/>
+      <c r="K52" s="16"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A53" s="27" t="s">
+      <c r="A53" s="18"/>
+      <c r="B53" s="18"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="23"/>
+      <c r="E53" s="23"/>
+      <c r="F53" s="8"/>
+      <c r="G53" s="9"/>
+      <c r="H53" s="9"/>
+      <c r="I53" s="9"/>
+      <c r="J53" s="10"/>
+      <c r="K53" s="10"/>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A54" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B53" s="28"/>
-      <c r="C53" s="28"/>
-      <c r="D53" s="28"/>
-      <c r="E53" s="20"/>
-      <c r="F53" s="11"/>
-      <c r="G53" s="27" t="s">
+      <c r="B54" s="44"/>
+      <c r="C54" s="44"/>
+      <c r="D54" s="44"/>
+      <c r="E54" s="20"/>
+      <c r="F54" s="11"/>
+      <c r="G54" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="H53" s="28"/>
-      <c r="I53" s="28"/>
-      <c r="J53" s="28"/>
-      <c r="K53" s="20"/>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A54" s="29" t="s">
+      <c r="H54" s="44"/>
+      <c r="I54" s="44"/>
+      <c r="J54" s="44"/>
+      <c r="K54" s="20"/>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A55" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="B54" s="28"/>
-      <c r="C54" s="28"/>
-      <c r="D54" s="28"/>
-      <c r="E54" s="21"/>
-      <c r="F54" s="11"/>
-      <c r="G54" s="29" t="s">
+      <c r="B55" s="44"/>
+      <c r="C55" s="44"/>
+      <c r="D55" s="44"/>
+      <c r="E55" s="21"/>
+      <c r="F55" s="11"/>
+      <c r="G55" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="H54" s="28"/>
-      <c r="I54" s="28"/>
-      <c r="J54" s="28"/>
-      <c r="K54" s="21"/>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A55" s="27" t="s">
+      <c r="H55" s="44"/>
+      <c r="I55" s="44"/>
+      <c r="J55" s="44"/>
+      <c r="K55" s="21"/>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A56" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="B55" s="28"/>
-      <c r="C55" s="28"/>
-      <c r="D55" s="28"/>
-      <c r="E55" s="20"/>
-      <c r="F55" s="11"/>
-      <c r="G55" s="27" t="s">
+      <c r="B56" s="44"/>
+      <c r="C56" s="44"/>
+      <c r="D56" s="44"/>
+      <c r="E56" s="20"/>
+      <c r="F56" s="11"/>
+      <c r="G56" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="H55" s="28"/>
-      <c r="I55" s="28"/>
-      <c r="J55" s="28"/>
-      <c r="K55" s="20"/>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A56" s="24" t="s">
+      <c r="H56" s="44"/>
+      <c r="I56" s="44"/>
+      <c r="J56" s="44"/>
+      <c r="K56" s="20"/>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A57" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="B57" s="44"/>
+      <c r="C57" s="44"/>
+      <c r="D57" s="44"/>
+      <c r="E57" s="20"/>
+      <c r="F57" s="11"/>
+      <c r="G57" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="H57" s="44"/>
+      <c r="I57" s="44"/>
+      <c r="J57" s="44"/>
+      <c r="K57" s="20"/>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A58" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="B56" s="25"/>
-      <c r="C56" s="25"/>
-      <c r="D56" s="25"/>
-      <c r="E56" s="26"/>
-      <c r="F56" s="22"/>
-      <c r="G56" s="24" t="s">
+      <c r="B58" s="46"/>
+      <c r="C58" s="46"/>
+      <c r="D58" s="46"/>
+      <c r="E58" s="47"/>
+      <c r="F58" s="22"/>
+      <c r="G58" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="H56" s="25"/>
-      <c r="I56" s="25"/>
-      <c r="J56" s="25"/>
-      <c r="K56" s="26"/>
+      <c r="H58" s="46"/>
+      <c r="I58" s="46"/>
+      <c r="J58" s="46"/>
+      <c r="K58" s="47"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="33">
+    <mergeCell ref="G58:K58"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="G54:J54"/>
+    <mergeCell ref="G55:J55"/>
+    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="G56:J56"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="G57:J57"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="G32:K32"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="G33:K33"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="G27:J27"/>
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="G16:K16"/>
     <mergeCell ref="A1:K1"/>
@@ -2498,28 +2562,6 @@
     <mergeCell ref="G3:K3"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="G4:K4"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="G44:K44"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="G28:K28"/>
-    <mergeCell ref="A31:E31"/>
-    <mergeCell ref="G31:K31"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="G32:K32"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="G27:J27"/>
-    <mergeCell ref="G56:K56"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="G53:J53"/>
-    <mergeCell ref="G54:J54"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="G55:J55"/>
-    <mergeCell ref="A56:E56"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>